<commit_message>
Match rate suggestions to pricing-rule conditions and price only the latest buy and sell ratings.
Profit stays empty when one side or the reporting FX rate is missing. Each side keeps its own chargeable quantity.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/po/12102026/LCMS_Consolidated_Change_Request_DEV_2026-10-12_v1.0_AC_Traceability.xlsx
+++ b/docs/po/12102026/LCMS_Consolidated_Change_Request_DEV_2026-10-12_v1.0_AC_Traceability.xlsx
@@ -685,7 +685,7 @@
       </c>
       <c r="F4" s="10" t="inlineStr">
         <is>
-          <t>Unit Published_wrong_route_is_not_selectable: Pass. Lý do «Không khớp tuyến».</t>
+          <t>API BillRateSuggestionApiTests.Suggestion_UsesRuleRoute: quy tắc SGN-DAD không được chọn khi Bill là SGN-HAN. Pass.</t>
         </is>
       </c>
     </row>
@@ -749,7 +749,7 @@
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>Unit Retired_card_cannot_be_selected: Pass. RatingContextResolver từ chối bảng giá ngừng sử dụng.</t>
+          <t>API cùng test: sau khi ngừng bảng giá, POST /api/ratings trả 409. Pass.</t>
         </is>
       </c>
     </row>
@@ -909,7 +909,7 @@
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
-          <t>BUY và SELL được phân loại riêng. Unit Buy_and_sell_are_classified_separately: Pass. Cách tính từng chiều vẫn do quy tắc của phiên bản đã chọn.</t>
+          <t>Mỗi chiều có ô khối lượng riêng. Chưa chụp màn hình.</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>Lợi nhuận chỉ hiện khi đủ hai chiều và reportingComplete. Chưa có Bill mẫu FX trên site.</t>
+          <t>API Margin_IsBuySellRatingsOnly: 1.000 và 1.800 VND cho lợi nhuận 800. Chỉ lấy hai lần tính mới nhất. Pass.</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
-          <t>expectedProfitView ẩn số khi thiếu tỷ giá, không thay bằng 0. Kiểm tra hàm trên Node: Pass.</t>
+          <t>API cùng test: chiều bán USD không có tỷ giá thì ReportingProfit null, FxMissing true. Pass.</t>
         </is>
       </c>
     </row>
@@ -1165,7 +1165,7 @@
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>Một chiều thì không hiện số lợi nhuận. Kiểm tra hàm expectedProfitView trên Node: Pass.</t>
+          <t>Unit One_side_does_not_show_profit: Pass. Không hiện số lợi nhuận.</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
-          <t>HOLD. ADR-0024 mục 3: màn tạo giữ tổng, không lưới dòng. W-K1 sau đó đã thêm lưới. Thiếu nguyên văn PO khớp AC này.</t>
+          <t>HOLD. Đã đọc CreateBillWorkspaceForm và validateCargoLines: dòng trống được bỏ, không bắt buộc cả kiện và container. Chưa có đối chiếu tổng dòng với tổng Bill. ADR-0024 mục 3 vẫn mâu thuẫn với lưới đang có.</t>
         </is>
       </c>
     </row>
@@ -1357,7 +1357,7 @@
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
-          <t>HOLD. Cùng nguồn ADR-0024 và W-K1. Không tự thiết kế.</t>
+          <t>HOLD. Cùng kết quả đọc form. Không suy ra số container từ số kiện trong validateCargoLines. Chưa chốt quy tắc đối chiếu tổng.</t>
         </is>
       </c>
     </row>
@@ -1966,12 +1966,12 @@
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
-          <t>Unit Published_wrong_route_is_not_selectable: Pass. Lý do «Không khớp tuyến».</t>
+          <t>API BillRateSuggestionApiTests.Suggestion_UsesRuleRoute: quy tắc SGN-DAD không được chọn khi Bill là SGN-HAN. Pass.</t>
         </is>
       </c>
       <c r="F4" s="10" t="inlineStr">
         <is>
-          <t>Một phần</t>
+          <t>Đạt API</t>
         </is>
       </c>
       <c r="G4" s="10" t="inlineStr">
@@ -2050,12 +2050,12 @@
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>Unit Retired_card_cannot_be_selected: Pass. RatingContextResolver từ chối bảng giá ngừng sử dụng.</t>
+          <t>API cùng test: sau khi ngừng bảng giá, POST /api/ratings trả 409. Pass.</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>Một phần</t>
+          <t>Đạt API</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
@@ -2260,12 +2260,12 @@
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>BUY và SELL được phân loại riêng. Unit Buy_and_sell_are_classified_separately: Pass. Cách tính từng chiều vẫn do quy tắc của phiên bản đã chọn.</t>
+          <t>Mỗi chiều có ô khối lượng riêng. Chưa chụp màn hình.</t>
         </is>
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
-          <t>Một phần</t>
+          <t>Đạt API</t>
         </is>
       </c>
       <c r="G11" s="10" t="inlineStr">
@@ -2428,12 +2428,12 @@
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>Lợi nhuận chỉ hiện khi đủ hai chiều và reportingComplete. Chưa có Bill mẫu FX trên site.</t>
+          <t>API Margin_IsBuySellRatingsOnly: 1.000 và 1.800 VND cho lợi nhuận 800. Chỉ lấy hai lần tính mới nhất. Pass.</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>Một phần</t>
+          <t>Đạt API</t>
         </is>
       </c>
       <c r="G15" s="10" t="inlineStr">
@@ -2470,12 +2470,12 @@
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>expectedProfitView ẩn số khi thiếu tỷ giá, không thay bằng 0. Kiểm tra hàm trên Node: Pass.</t>
+          <t>API cùng test: chiều bán USD không có tỷ giá thì ReportingProfit null, FxMissing true. Pass.</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
-          <t>Một phần</t>
+          <t>Đạt API</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
@@ -2596,12 +2596,12 @@
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>Một chiều thì không hiện số lợi nhuận. Kiểm tra hàm expectedProfitView trên Node: Pass.</t>
+          <t>Unit One_side_does_not_show_profit: Pass. Không hiện số lợi nhuận.</t>
         </is>
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>Một phần</t>
+          <t>Đạt API</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
-          <t>HOLD. ADR-0024 mục 3: màn tạo giữ tổng, không lưới dòng. W-K1 sau đó đã thêm lưới. Thiếu nguyên văn PO khớp AC này.</t>
+          <t>HOLD. Đã đọc CreateBillWorkspaceForm và validateCargoLines: dòng trống được bỏ, không bắt buộc cả kiện và container. Chưa có đối chiếu tổng dòng với tổng Bill. ADR-0024 mục 3 vẫn mâu thuẫn với lưới đang có.</t>
         </is>
       </c>
       <c r="F24" s="10" t="inlineStr">
@@ -2848,7 +2848,7 @@
       </c>
       <c r="E25" s="10" t="inlineStr">
         <is>
-          <t>HOLD. Cùng nguồn ADR-0024 và W-K1. Không tự thiết kế.</t>
+          <t>HOLD. Cùng kết quả đọc form. Không suy ra số container từ số kiện trong validateCargoLines. Chưa chốt quy tắc đối chiếu tổng.</t>
         </is>
       </c>
       <c r="F25" s="10" t="inlineStr">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>ADR-0024 mục 3 khác W-K1. Chưa sửa màn Bill</t>
+          <t>Đã đọc form tạo Bill. Dòng kiện không bắt buộc. Chưa có rule đối chiếu tổng. Vẫn HOLD.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hide expected rating margin unless the user can read both cost and revenue.
A cost-only accountant no longer receives the sell rating or a profit figure.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/po/12102026/LCMS_Consolidated_Change_Request_DEV_2026-10-12_v1.0_AC_Traceability.xlsx
+++ b/docs/po/12102026/LCMS_Consolidated_Change_Request_DEV_2026-10-12_v1.0_AC_Traceability.xlsx
@@ -1037,7 +1037,7 @@
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>API Margin_IsBuySellRatingsOnly: 1.000 và 1.800 VND cho lợi nhuận 800. Chỉ lấy hai lần tính mới nhất. Pass.</t>
+          <t>API Margin_IsBuySellRatingsOnly: 1.000 và 1.800 VND cho lợi nhuận 800. Chỉ lấy hai lần tính mới nhất. Pass. API CostAccountant_DoesNotSeeSellRatingOrProfit Pass: kế toán chi phí không nhận số chiều bán, không nhận lợi nhuận, không thấy lần tính giá bán. Chưa có ảnh trên site đang chạy.</t>
         </is>
       </c>
     </row>
@@ -2428,7 +2428,7 @@
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>API Margin_IsBuySellRatingsOnly: 1.000 và 1.800 VND cho lợi nhuận 800. Chỉ lấy hai lần tính mới nhất. Pass.</t>
+          <t>API Margin_IsBuySellRatingsOnly: 1.000 và 1.800 VND cho lợi nhuận 800. Chỉ lấy hai lần tính mới nhất. Pass. API CostAccountant_DoesNotSeeSellRatingOrProfit Pass: kế toán chi phí không nhận số chiều bán, không nhận lợi nhuận, không thấy lần tính giá bán. Chưa có ảnh trên site đang chạy.</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Keep Bill create on totals only, per the locked ADR-0024 decision.
An air bill saves without package lines, and a blank package count is not stored as one piece.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/po/12102026/LCMS_Consolidated_Change_Request_DEV_2026-10-12_v1.0_AC_Traceability.xlsx
+++ b/docs/po/12102026/LCMS_Consolidated_Change_Request_DEV_2026-10-12_v1.0_AC_Traceability.xlsx
@@ -1325,7 +1325,7 @@
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
-          <t>HOLD. Đã đọc CreateBillWorkspaceForm và validateCargoLines: dòng trống được bỏ, không bắt buộc cả kiện và container. Chưa có đối chiếu tổng dòng với tổng Bill. ADR-0024 mục 3 vẫn mâu thuẫn với lưới đang có.</t>
+          <t>PO chốt phương án 1 theo ADR-0024. Màn tạo Bill chỉ còn số tổng, không còn lưới kiện/container. API BillCreateTotalsTests.Air_bill_saves_without_package_lines_and_keeps_entered_totals Pass: Bill AIR không có số kiện vẫn lưu, trọng lượng và thể tích đã nhập được giữ. Chưa có ảnh trên site đang chạy.</t>
         </is>
       </c>
     </row>
@@ -1357,7 +1357,7 @@
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
-          <t>HOLD. Cùng kết quả đọc form. Không suy ra số container từ số kiện trong validateCargoLines. Chưa chốt quy tắc đối chiếu tổng.</t>
+          <t>PO chốt màn tạo không quản lý từng kiện nên không đối chiếu tổng dòng. Số tổng đã nhập là đầu vào tính giá. Cùng test Pass. Không đổi quy tắc trọng lượng tính cước và kiểm soát Rating.</t>
         </is>
       </c>
     </row>
@@ -2806,12 +2806,12 @@
       </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
-          <t>HOLD. Đã đọc CreateBillWorkspaceForm và validateCargoLines: dòng trống được bỏ, không bắt buộc cả kiện và container. Chưa có đối chiếu tổng dòng với tổng Bill. ADR-0024 mục 3 vẫn mâu thuẫn với lưới đang có.</t>
+          <t>PO chốt phương án 1 theo ADR-0024. Màn tạo Bill chỉ còn số tổng, không còn lưới kiện/container. API BillCreateTotalsTests.Air_bill_saves_without_package_lines_and_keeps_entered_totals Pass: Bill AIR không có số kiện vẫn lưu, trọng lượng và thể tích đã nhập được giữ. Chưa có ảnh trên site đang chạy.</t>
         </is>
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>Đạt phương án 1</t>
         </is>
       </c>
       <c r="G24" s="10" t="inlineStr">
@@ -2848,12 +2848,12 @@
       </c>
       <c r="E25" s="10" t="inlineStr">
         <is>
-          <t>HOLD. Cùng kết quả đọc form. Không suy ra số container từ số kiện trong validateCargoLines. Chưa chốt quy tắc đối chiếu tổng.</t>
+          <t>PO chốt màn tạo không quản lý từng kiện nên không đối chiếu tổng dòng. Số tổng đã nhập là đầu vào tính giá. Cùng test Pass. Không đổi quy tắc trọng lượng tính cước và kiểm soát Rating.</t>
         </is>
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>Đạt phương án 1</t>
         </is>
       </c>
       <c r="G25" s="10" t="inlineStr">
@@ -3214,12 +3214,12 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>Đã triển khai phương án 1</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Đã đọc form tạo Bill. Dòng kiện không bắt buộc. Chưa có rule đối chiếu tổng. Vẫn HOLD.</t>
+          <t>Màn tạo Bill chỉ số tổng. BillCreateTotalsTests Pass. Chưa có ảnh site.</t>
         </is>
       </c>
     </row>

</xml_diff>